<commit_message>
ToDos + Plan Obsidian
</commit_message>
<xml_diff>
--- a/biomechanics/execution/exercise_kinematics.xlsx
+++ b/biomechanics/execution/exercise_kinematics.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kubis\Projekte\GYM_APP\biomechanics\execution\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{977763D3-6EBC-40A4-948E-75F58F4B3160}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB9056FD-EBAC-40A2-A6A4-71DDE22FEB48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Uebungen" sheetId="1" r:id="rId1"/>

</xml_diff>